<commit_message>
parameters file now date agnostic to prepare for forthcoming July2026 BOLDistilled release
</commit_message>
<xml_diff>
--- a/workdir/parameters.xlsx
+++ b/workdir/parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickbard/Desktop/CBG/BIP/wkdir/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickbard/Desktop/CBG/BIP/workdir/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{691E9077-8EB0-9743-BCBB-3115653A8C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2599BCA2-D1BF-AC42-9AA8-F64E0BF74ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30060" yWindow="2480" windowWidth="28860" windowHeight="15700" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30060" yWindow="4200" windowWidth="28860" windowHeight="15700" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -1593,7 +1593,7 @@
     <t>Max amplicon length</t>
   </si>
   <si>
-    <t>BOLDistilled_COI_Apr2026</t>
+    <t>BOLDistilled_COI_</t>
   </si>
 </sst>
 </file>
@@ -8865,14 +8865,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7e688c01-aefd-4b2f-9d3c-b02cde5b1282">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f4163dc9-7f99-4634-8785-23aba72f7f8a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9111,21 +9109,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7e688c01-aefd-4b2f-9d3c-b02cde5b1282">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f4163dc9-7f99-4634-8785-23aba72f7f8a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19D4B927-2C05-41EC-B7D9-143B0AC62050}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C431F7D-3CA3-4AE8-9186-312DA139C36E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="7e688c01-aefd-4b2f-9d3c-b02cde5b1282"/>
-    <ds:schemaRef ds:uri="f4163dc9-7f99-4634-8785-23aba72f7f8a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9150,9 +9147,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C431F7D-3CA3-4AE8-9186-312DA139C36E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19D4B927-2C05-41EC-B7D9-143B0AC62050}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="7e688c01-aefd-4b2f-9d3c-b02cde5b1282"/>
+    <ds:schemaRef ds:uri="f4163dc9-7f99-4634-8785-23aba72f7f8a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>